<commit_message>
Cambio en archivos para reunión 3 con la super, se agrega carpeta y archivos para comité de ética
</commit_message>
<xml_diff>
--- a/Modelo/datos/Raw_Data/Matriz_de_Adyacencia_Pensiones_validada_NO_TOCAR.xlsx
+++ b/Modelo/datos/Raw_Data/Matriz_de_Adyacencia_Pensiones_validada_NO_TOCAR.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/21a7d57e8591b932/Escritorio/CICS/2025/Tesis/Objetivos de Aprendizaje/Modelo/datos/Raw_Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="651" documentId="8_{00D88C31-2993-4F88-955D-B3AEA2AC3E47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{527E32A8-3B6A-4EDB-A596-CD9A7D230C11}"/>
+  <xr:revisionPtr revIDLastSave="654" documentId="8_{00D88C31-2993-4F88-955D-B3AEA2AC3E47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{097920CD-50F3-44A4-9CD3-B49AA71A0C22}"/>
   <bookViews>
-    <workbookView xWindow="43080" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E85862A8-A9B5-4BB7-B4AF-3D0252E6C1A3}"/>
+    <workbookView xWindow="14303" yWindow="-1155" windowWidth="21795" windowHeight="12975" xr2:uid="{E85862A8-A9B5-4BB7-B4AF-3D0252E6C1A3}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -295,8 +295,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -374,7 +382,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1417,34 +1425,34 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7DD69CEB-FB4B-428B-8D1B-77C5ED66F830}">
   <dimension ref="A1:BU73"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="27.59765625" customWidth="1"/>
-    <col min="3" max="4" width="11.59765625" customWidth="1"/>
-    <col min="5" max="6" width="11.3984375" customWidth="1"/>
-    <col min="7" max="7" width="10.86328125" customWidth="1"/>
-    <col min="8" max="13" width="11.3984375" customWidth="1"/>
-    <col min="14" max="14" width="13.86328125" customWidth="1"/>
-    <col min="15" max="19" width="11.3984375" customWidth="1"/>
-    <col min="20" max="20" width="10.86328125" customWidth="1"/>
-    <col min="21" max="21" width="11.3984375" customWidth="1"/>
-    <col min="22" max="22" width="10.86328125" customWidth="1"/>
-    <col min="23" max="26" width="11.3984375" customWidth="1"/>
-    <col min="27" max="28" width="10.86328125" customWidth="1"/>
-    <col min="29" max="29" width="13.265625" customWidth="1"/>
-    <col min="30" max="30" width="13.59765625" customWidth="1"/>
-    <col min="31" max="34" width="11.3984375" customWidth="1"/>
-    <col min="35" max="35" width="20.59765625" bestFit="1" customWidth="1"/>
-    <col min="36" max="47" width="11.3984375" customWidth="1"/>
-    <col min="48" max="48" width="13.86328125" customWidth="1"/>
-    <col min="49" max="61" width="11.3984375" customWidth="1"/>
-    <col min="62" max="68" width="10.86328125" customWidth="1"/>
-    <col min="69" max="72" width="11.3984375" customWidth="1"/>
-    <col min="73" max="74" width="10.86328125" customWidth="1"/>
-    <col min="75" max="75" width="11.3984375" customWidth="1"/>
+    <col min="2" max="2" width="27.5703125" customWidth="1"/>
+    <col min="3" max="4" width="11.5703125" customWidth="1"/>
+    <col min="5" max="6" width="11.42578125" customWidth="1"/>
+    <col min="7" max="7" width="10.85546875" customWidth="1"/>
+    <col min="8" max="13" width="11.42578125" customWidth="1"/>
+    <col min="14" max="14" width="13.85546875" customWidth="1"/>
+    <col min="15" max="19" width="11.42578125" customWidth="1"/>
+    <col min="20" max="20" width="10.85546875" customWidth="1"/>
+    <col min="21" max="21" width="11.42578125" customWidth="1"/>
+    <col min="22" max="22" width="10.85546875" customWidth="1"/>
+    <col min="23" max="26" width="11.42578125" customWidth="1"/>
+    <col min="27" max="28" width="10.85546875" customWidth="1"/>
+    <col min="29" max="29" width="13.28515625" customWidth="1"/>
+    <col min="30" max="30" width="13.5703125" customWidth="1"/>
+    <col min="31" max="34" width="11.42578125" customWidth="1"/>
+    <col min="35" max="35" width="20.5703125" bestFit="1" customWidth="1"/>
+    <col min="36" max="47" width="11.42578125" customWidth="1"/>
+    <col min="48" max="48" width="13.85546875" customWidth="1"/>
+    <col min="49" max="61" width="11.42578125" customWidth="1"/>
+    <col min="62" max="68" width="10.85546875" customWidth="1"/>
+    <col min="69" max="72" width="11.42578125" customWidth="1"/>
+    <col min="73" max="74" width="10.85546875" customWidth="1"/>
+    <col min="75" max="75" width="11.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:73" x14ac:dyDescent="0.25">
       <c r="C1">
         <v>1</v>
       </c>
@@ -1659,7 +1667,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="2" spans="1:73" ht="57" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:73" ht="60" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>59</v>
       </c>
@@ -1877,14 +1885,14 @@
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3" t="s">
         <v>81</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="8">
         <v>1</v>
       </c>
       <c r="G3" s="1"/>
@@ -1915,13 +1923,13 @@
       <c r="AF3" s="1"/>
       <c r="AG3" s="1"/>
       <c r="AL3" s="1"/>
-      <c r="AM3" s="8"/>
-      <c r="AN3" s="8"/>
-      <c r="AO3" s="8"/>
-      <c r="AP3" s="8"/>
-      <c r="AQ3" s="8"/>
-      <c r="AR3" s="8"/>
-      <c r="AS3" s="8"/>
+      <c r="AM3" s="1"/>
+      <c r="AN3" s="1"/>
+      <c r="AO3" s="1"/>
+      <c r="AP3" s="1"/>
+      <c r="AQ3" s="1"/>
+      <c r="AR3" s="1"/>
+      <c r="AS3" s="1"/>
       <c r="AT3" s="1"/>
       <c r="AU3" s="1"/>
       <c r="AV3" s="1"/>
@@ -1951,7 +1959,7 @@
       <c r="BT3" s="1"/>
       <c r="BU3" s="1"/>
     </row>
-    <row r="4" spans="1:73" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="4" spans="1:73" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2</v>
       </c>
@@ -1960,11 +1968,15 @@
       </c>
       <c r="E4" s="1"/>
       <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
+      <c r="H4" s="1">
+        <v>1</v>
+      </c>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
-      <c r="L4" s="1"/>
+      <c r="L4" s="1">
+        <v>1</v>
+      </c>
       <c r="M4" s="1"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
@@ -1987,13 +1999,13 @@
       <c r="AF4" s="1"/>
       <c r="AG4" s="1"/>
       <c r="AL4" s="1"/>
-      <c r="AM4" s="8"/>
-      <c r="AN4" s="8"/>
-      <c r="AO4" s="8"/>
-      <c r="AP4" s="8"/>
-      <c r="AQ4" s="8"/>
-      <c r="AR4" s="8"/>
-      <c r="AS4" s="8"/>
+      <c r="AM4" s="1"/>
+      <c r="AN4" s="1"/>
+      <c r="AO4" s="1"/>
+      <c r="AP4" s="1"/>
+      <c r="AQ4" s="1"/>
+      <c r="AR4" s="1"/>
+      <c r="AS4" s="1"/>
       <c r="AT4" s="1"/>
       <c r="AU4" s="1"/>
       <c r="AV4" s="1"/>
@@ -2023,7 +2035,7 @@
       <c r="BT4" s="1"/>
       <c r="BU4" s="1"/>
     </row>
-    <row r="5" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>3</v>
       </c>
@@ -2178,7 +2190,7 @@
       </c>
       <c r="BU5" s="2"/>
     </row>
-    <row r="6" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>4</v>
       </c>
@@ -2210,7 +2222,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>5</v>
       </c>
@@ -2218,7 +2230,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="8" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>6</v>
       </c>
@@ -2289,7 +2301,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>7</v>
       </c>
@@ -2360,7 +2372,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:73" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="10" spans="1:73" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>8</v>
       </c>
@@ -2380,7 +2392,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>9</v>
       </c>
@@ -2491,7 +2503,7 @@
       <c r="BT11" s="2"/>
       <c r="BU11" s="2"/>
     </row>
-    <row r="12" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>10</v>
       </c>
@@ -2562,7 +2574,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>11</v>
       </c>
@@ -2579,7 +2591,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>12</v>
       </c>
@@ -2587,7 +2599,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="15" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>13</v>
       </c>
@@ -2598,7 +2610,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:73" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="16" spans="1:73" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>14</v>
       </c>
@@ -2689,7 +2701,7 @@
       <c r="BT16" s="3"/>
       <c r="BU16" s="3"/>
     </row>
-    <row r="17" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>15</v>
       </c>
@@ -2798,7 +2810,7 @@
       <c r="BT17" s="2"/>
       <c r="BU17" s="2"/>
     </row>
-    <row r="18" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>16</v>
       </c>
@@ -2818,7 +2830,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>17</v>
       </c>
@@ -2847,7 +2859,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>18</v>
       </c>
@@ -2855,7 +2867,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="21" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>19</v>
       </c>
@@ -2869,7 +2881,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>20</v>
       </c>
@@ -2877,7 +2889,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="23" spans="1:73" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="23" spans="1:73" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>21</v>
       </c>
@@ -2900,7 +2912,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>22</v>
       </c>
@@ -2981,7 +2993,7 @@
       <c r="BT24" s="2"/>
       <c r="BU24" s="2"/>
     </row>
-    <row r="25" spans="1:73" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="25" spans="1:73" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>23</v>
       </c>
@@ -2989,7 +3001,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="26" spans="1:73" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="26" spans="1:73" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>24</v>
       </c>
@@ -3068,7 +3080,7 @@
       <c r="BT26" s="2"/>
       <c r="BU26" s="2"/>
     </row>
-    <row r="27" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>25</v>
       </c>
@@ -3147,7 +3159,7 @@
       <c r="BT27" s="2"/>
       <c r="BU27" s="2"/>
     </row>
-    <row r="28" spans="1:73" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="28" spans="1:73" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>26</v>
       </c>
@@ -3228,7 +3240,7 @@
       <c r="BT28" s="3"/>
       <c r="BU28" s="3"/>
     </row>
-    <row r="29" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>27</v>
       </c>
@@ -3309,7 +3321,7 @@
       <c r="BT29" s="2"/>
       <c r="BU29" s="2"/>
     </row>
-    <row r="30" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>28</v>
       </c>
@@ -3317,7 +3329,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="31" spans="1:73" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="31" spans="1:73" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>29</v>
       </c>
@@ -3422,7 +3434,7 @@
       <c r="BT31" s="3"/>
       <c r="BU31" s="3"/>
     </row>
-    <row r="32" spans="1:73" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="32" spans="1:73" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>30</v>
       </c>
@@ -3509,7 +3521,7 @@
       <c r="BT32" s="2"/>
       <c r="BU32" s="2"/>
     </row>
-    <row r="33" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>31</v>
       </c>
@@ -3596,7 +3608,7 @@
       <c r="BT33" s="2"/>
       <c r="BU33" s="2"/>
     </row>
-    <row r="34" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>32</v>
       </c>
@@ -3631,7 +3643,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>33</v>
       </c>
@@ -3651,7 +3663,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>34</v>
       </c>
@@ -3674,7 +3686,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>35</v>
       </c>
@@ -3694,7 +3706,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:73" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="38" spans="1:73" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>36</v>
       </c>
@@ -3702,7 +3714,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="39" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>37</v>
       </c>
@@ -3833,7 +3845,7 @@
       <c r="BT39" s="2"/>
       <c r="BU39" s="2"/>
     </row>
-    <row r="40" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>38</v>
       </c>
@@ -3850,7 +3862,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>39</v>
       </c>
@@ -3891,7 +3903,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:73" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="42" spans="1:73" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>40</v>
       </c>
@@ -3980,7 +3992,7 @@
       <c r="BT42" s="3"/>
       <c r="BU42" s="3"/>
     </row>
-    <row r="43" spans="1:73" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:73" ht="30" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>41</v>
       </c>
@@ -4002,7 +4014,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>42</v>
       </c>
@@ -4022,7 +4034,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:73" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="45" spans="1:73" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>43</v>
       </c>
@@ -4042,7 +4054,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:73" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="46" spans="1:73" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>44</v>
       </c>
@@ -4163,7 +4175,7 @@
       <c r="BT46" s="5"/>
       <c r="BU46" s="5"/>
     </row>
-    <row r="47" spans="1:73" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="47" spans="1:73" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>45</v>
       </c>
@@ -4248,7 +4260,7 @@
       <c r="BT47" s="3"/>
       <c r="BU47" s="3"/>
     </row>
-    <row r="48" spans="1:73" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="48" spans="1:73" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>46</v>
       </c>
@@ -4335,7 +4347,7 @@
       <c r="BT48" s="2"/>
       <c r="BU48" s="2"/>
     </row>
-    <row r="49" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>47</v>
       </c>
@@ -4442,7 +4454,7 @@
       <c r="BT49" s="2"/>
       <c r="BU49" s="2"/>
     </row>
-    <row r="50" spans="1:73" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="50" spans="1:73" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>48</v>
       </c>
@@ -4521,7 +4533,7 @@
       <c r="BT50" s="3"/>
       <c r="BU50" s="3"/>
     </row>
-    <row r="51" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>49</v>
       </c>
@@ -4630,7 +4642,7 @@
       <c r="BT51" s="2"/>
       <c r="BU51" s="2"/>
     </row>
-    <row r="52" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>50</v>
       </c>
@@ -4653,7 +4665,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>51</v>
       </c>
@@ -4667,7 +4679,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:73" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="54" spans="1:73" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>52</v>
       </c>
@@ -4752,7 +4764,7 @@
       <c r="BT54" s="3"/>
       <c r="BU54" s="3"/>
     </row>
-    <row r="55" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>53</v>
       </c>
@@ -4855,7 +4867,7 @@
       <c r="BT55" s="2"/>
       <c r="BU55" s="2"/>
     </row>
-    <row r="56" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>54</v>
       </c>
@@ -4869,7 +4881,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:73" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="57" spans="1:73" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>55</v>
       </c>
@@ -4910,7 +4922,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:73" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="58" spans="1:73" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>56</v>
       </c>
@@ -4989,7 +5001,7 @@
       <c r="BT58" s="2"/>
       <c r="BU58" s="2"/>
     </row>
-    <row r="59" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>57</v>
       </c>
@@ -5074,7 +5086,7 @@
       <c r="BT59" s="2"/>
       <c r="BU59" s="2"/>
     </row>
-    <row r="60" spans="1:73" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="60" spans="1:73" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>58</v>
       </c>
@@ -5155,7 +5167,7 @@
       <c r="BT60" s="3"/>
       <c r="BU60" s="3"/>
     </row>
-    <row r="61" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>59</v>
       </c>
@@ -5163,7 +5175,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="62" spans="1:73" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="62" spans="1:73" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>60</v>
       </c>
@@ -5246,7 +5258,7 @@
       <c r="BT62" s="3"/>
       <c r="BU62" s="3"/>
     </row>
-    <row r="63" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>61</v>
       </c>
@@ -5327,7 +5339,7 @@
       <c r="BT63" s="2"/>
       <c r="BU63" s="2"/>
     </row>
-    <row r="64" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>62</v>
       </c>
@@ -5350,7 +5362,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:73" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="65" spans="1:73" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>63</v>
       </c>
@@ -5358,7 +5370,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="66" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>64</v>
       </c>
@@ -5437,7 +5449,7 @@
       <c r="BT66" s="2"/>
       <c r="BU66" s="2"/>
     </row>
-    <row r="67" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="67" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>65</v>
       </c>
@@ -5445,7 +5457,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="68" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="68" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>66</v>
       </c>
@@ -5453,7 +5465,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="69" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="69" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>67</v>
       </c>
@@ -5464,7 +5476,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:73" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="70" spans="1:73" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>68</v>
       </c>
@@ -5490,7 +5502,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:73" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="71" spans="1:73" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>69</v>
       </c>
@@ -5583,7 +5595,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="72" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>70</v>
       </c>
@@ -5668,7 +5680,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:73" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="73" spans="1:73" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>71</v>
       </c>
@@ -5806,8 +5818,8 @@
     <cfRule type="duplicateValues" dxfId="50" priority="1590"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B37:D37">
-    <cfRule type="duplicateValues" dxfId="49" priority="1"/>
-    <cfRule type="duplicateValues" dxfId="48" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="49" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="48" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B39:D46">
     <cfRule type="duplicateValues" dxfId="47" priority="1591"/>
@@ -5819,8 +5831,8 @@
     <cfRule type="duplicateValues" dxfId="45" priority="1593"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B49:D52">
-    <cfRule type="duplicateValues" dxfId="44" priority="1568"/>
-    <cfRule type="duplicateValues" dxfId="43" priority="1570"/>
+    <cfRule type="duplicateValues" dxfId="44" priority="1570"/>
+    <cfRule type="duplicateValues" dxfId="43" priority="1568"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B53:D53">
     <cfRule type="duplicateValues" dxfId="42" priority="1594"/>
@@ -5862,19 +5874,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34F02EE0-40BA-4311-B39A-384F2CBD26CC}">
   <dimension ref="A1:BT72"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="27.59765625" customWidth="1"/>
-    <col min="32" max="32" width="13.86328125" customWidth="1"/>
-    <col min="53" max="53" width="13.86328125" customWidth="1"/>
-    <col min="57" max="60" width="10.86328125" customWidth="1"/>
-    <col min="61" max="61" width="13.59765625" customWidth="1"/>
-    <col min="62" max="62" width="13.265625" customWidth="1"/>
-    <col min="63" max="63" width="13.3984375" customWidth="1"/>
-    <col min="64" max="73" width="10.86328125" customWidth="1"/>
+    <col min="1" max="1" width="27.5703125" customWidth="1"/>
+    <col min="32" max="32" width="13.85546875" customWidth="1"/>
+    <col min="53" max="53" width="13.85546875" customWidth="1"/>
+    <col min="57" max="60" width="10.85546875" customWidth="1"/>
+    <col min="61" max="61" width="13.5703125" customWidth="1"/>
+    <col min="62" max="62" width="13.28515625" customWidth="1"/>
+    <col min="63" max="63" width="13.42578125" customWidth="1"/>
+    <col min="64" max="73" width="10.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:72" ht="57.4" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:72" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -6089,7 +6101,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="2" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>60</v>
       </c>
@@ -6259,7 +6271,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>61</v>
       </c>
@@ -6306,7 +6318,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>35</v>
       </c>
@@ -6344,7 +6356,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>1</v>
       </c>
@@ -6373,7 +6385,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:72" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="6" spans="1:72" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -6393,7 +6405,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>3</v>
       </c>
@@ -6505,7 +6517,7 @@
       </c>
       <c r="BT7" s="2"/>
     </row>
-    <row r="8" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -6597,7 +6609,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -6650,7 +6662,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>6</v>
       </c>
@@ -6667,7 +6679,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>7</v>
       </c>
@@ -6696,7 +6708,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:72" ht="28.9" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="12" spans="1:72" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>8</v>
       </c>
@@ -6788,7 +6800,7 @@
       <c r="BS12" s="3"/>
       <c r="BT12" s="3"/>
     </row>
-    <row r="13" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>9</v>
       </c>
@@ -6908,7 +6920,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>10</v>
       </c>
@@ -6988,7 +7000,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>11</v>
       </c>
@@ -7065,7 +7077,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>12</v>
       </c>
@@ -7082,7 +7094,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>13</v>
       </c>
@@ -7102,12 +7114,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="19" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>63</v>
       </c>
@@ -7166,7 +7178,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>15</v>
       </c>
@@ -7192,7 +7204,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:72" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="21" spans="1:72" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
         <v>64</v>
       </c>
@@ -7272,7 +7284,7 @@
       <c r="BS21" s="3"/>
       <c r="BT21" s="3"/>
     </row>
-    <row r="22" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>16</v>
       </c>
@@ -7380,12 +7392,12 @@
       <c r="BS22" s="2"/>
       <c r="BT22" s="2"/>
     </row>
-    <row r="23" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="24" spans="1:72" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="24" spans="1:72" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
         <v>69</v>
       </c>
@@ -7465,7 +7477,7 @@
       <c r="BS24" s="3"/>
       <c r="BT24" s="3"/>
     </row>
-    <row r="25" spans="1:72" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="25" spans="1:72" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>18</v>
       </c>
@@ -7577,7 +7589,7 @@
       <c r="BS25" s="2"/>
       <c r="BT25" s="2"/>
     </row>
-    <row r="26" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>19</v>
       </c>
@@ -7685,7 +7697,7 @@
       <c r="BS26" s="2"/>
       <c r="BT26" s="2"/>
     </row>
-    <row r="27" spans="1:72" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="27" spans="1:72" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
         <v>65</v>
       </c>
@@ -7761,7 +7773,7 @@
       <c r="BS27" s="3"/>
       <c r="BT27" s="3"/>
     </row>
-    <row r="28" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>20</v>
       </c>
@@ -7845,7 +7857,7 @@
       <c r="BS28" s="2"/>
       <c r="BT28" s="2"/>
     </row>
-    <row r="29" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>21</v>
       </c>
@@ -7853,7 +7865,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:72" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="30" spans="1:72" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
         <v>22</v>
       </c>
@@ -7929,7 +7941,7 @@
       <c r="BS30" s="3"/>
       <c r="BT30" s="3"/>
     </row>
-    <row r="31" spans="1:72" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="31" spans="1:72" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>23</v>
       </c>
@@ -8013,7 +8025,7 @@
       <c r="BS31" s="2"/>
       <c r="BT31" s="2"/>
     </row>
-    <row r="32" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>24</v>
       </c>
@@ -8101,7 +8113,7 @@
       <c r="BS32" s="2"/>
       <c r="BT32" s="2"/>
     </row>
-    <row r="33" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>25</v>
       </c>
@@ -8124,7 +8136,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:72" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="34" spans="1:72" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>26</v>
       </c>
@@ -8144,7 +8156,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>27</v>
       </c>
@@ -8234,7 +8246,7 @@
       <c r="BS35" s="2"/>
       <c r="BT35" s="2"/>
     </row>
-    <row r="36" spans="1:72" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="36" spans="1:72" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="3" t="s">
         <v>73</v>
       </c>
@@ -8316,7 +8328,7 @@
       <c r="BS36" s="3"/>
       <c r="BT36" s="3"/>
     </row>
-    <row r="37" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>28</v>
       </c>
@@ -8404,7 +8416,7 @@
       <c r="BS37" s="2"/>
       <c r="BT37" s="2"/>
     </row>
-    <row r="38" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>29</v>
       </c>
@@ -8427,7 +8439,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>30</v>
       </c>
@@ -8435,7 +8447,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:72" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="40" spans="1:72" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="3" t="s">
         <v>31</v>
       </c>
@@ -8519,7 +8531,7 @@
       <c r="BS40" s="3"/>
       <c r="BT40" s="3"/>
     </row>
-    <row r="41" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>32</v>
       </c>
@@ -8533,7 +8545,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>33</v>
       </c>
@@ -8547,7 +8559,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:72" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="43" spans="1:72" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>70</v>
       </c>
@@ -8561,7 +8573,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:72" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="44" spans="1:72" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="5" t="s">
         <v>34</v>
       </c>
@@ -8647,7 +8659,7 @@
       <c r="BS44" s="5"/>
       <c r="BT44" s="5"/>
     </row>
-    <row r="45" spans="1:72" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="45" spans="1:72" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="3" t="s">
         <v>71</v>
       </c>
@@ -8741,7 +8753,7 @@
       <c r="BS45" s="3"/>
       <c r="BT45" s="3"/>
     </row>
-    <row r="46" spans="1:72" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="46" spans="1:72" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>44</v>
       </c>
@@ -8833,7 +8845,7 @@
       <c r="BS46" s="2"/>
       <c r="BT46" s="2"/>
     </row>
-    <row r="47" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>36</v>
       </c>
@@ -8917,7 +8929,7 @@
       <c r="BS47" s="2"/>
       <c r="BT47" s="2"/>
     </row>
-    <row r="48" spans="1:72" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="48" spans="1:72" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="3" t="s">
         <v>66</v>
       </c>
@@ -8997,7 +9009,7 @@
       <c r="BS48" s="3"/>
       <c r="BT48" s="3"/>
     </row>
-    <row r="49" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>37</v>
       </c>
@@ -9083,12 +9095,12 @@
       <c r="BS49" s="2"/>
       <c r="BT49" s="2"/>
     </row>
-    <row r="50" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="51" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>39</v>
       </c>
@@ -9096,7 +9108,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:72" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="52" spans="1:72" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="3" t="s">
         <v>40</v>
       </c>
@@ -9172,7 +9184,7 @@
       <c r="BS52" s="3"/>
       <c r="BT52" s="3"/>
     </row>
-    <row r="53" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>41</v>
       </c>
@@ -9248,7 +9260,7 @@
       <c r="BS53" s="2"/>
       <c r="BT53" s="2"/>
     </row>
-    <row r="54" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>72</v>
       </c>
@@ -9256,7 +9268,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:72" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="55" spans="1:72" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>42</v>
       </c>
@@ -9267,7 +9279,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:72" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="56" spans="1:72" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
         <v>43</v>
       </c>
@@ -9353,7 +9365,7 @@
       <c r="BS56" s="2"/>
       <c r="BT56" s="2"/>
     </row>
-    <row r="57" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>45</v>
       </c>
@@ -9429,7 +9441,7 @@
       <c r="BS57" s="2"/>
       <c r="BT57" s="2"/>
     </row>
-    <row r="58" spans="1:72" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="58" spans="1:72" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="3" t="s">
         <v>46</v>
       </c>
@@ -9505,12 +9517,12 @@
       <c r="BS58" s="3"/>
       <c r="BT58" s="3"/>
     </row>
-    <row r="59" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="60" spans="1:72" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="60" spans="1:72" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="3" t="s">
         <v>48</v>
       </c>
@@ -9588,7 +9600,7 @@
       <c r="BS60" s="3"/>
       <c r="BT60" s="3"/>
     </row>
-    <row r="61" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
         <v>49</v>
       </c>
@@ -9666,7 +9678,7 @@
       <c r="BS61" s="2"/>
       <c r="BT61" s="2"/>
     </row>
-    <row r="62" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>50</v>
       </c>
@@ -9674,17 +9686,17 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="64" spans="1:72" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="64" spans="1:72" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="65" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
         <v>67</v>
       </c>
@@ -9770,27 +9782,27 @@
       <c r="BS65" s="2"/>
       <c r="BT65" s="2"/>
     </row>
-    <row r="66" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="67" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="67" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="68" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="68" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="69" spans="1:72" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="69" spans="1:72" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="70" spans="1:72" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="70" spans="1:72" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
         <v>57</v>
       </c>
@@ -9872,7 +9884,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:72" x14ac:dyDescent="0.45">
+    <row r="71" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
         <v>58</v>
       </c>
@@ -9948,7 +9960,7 @@
       <c r="BS71" s="2"/>
       <c r="BT71" s="2"/>
     </row>
-    <row r="72" spans="1:72" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="72" spans="1:72" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A72" s="3" t="s">
         <v>68</v>
       </c>

</xml_diff>